<commit_message>
Revisi halaman: Medan tampil di Semua cabang, redaksi disederhanakan, tiga bagian Gap dihapus
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LYw4Jj7es2XsgtZASqqWXa
</commit_message>
<xml_diff>
--- a/dist/Peta_Proses_Audit_SOP_Review.xlsx
+++ b/dist/Peta_Proses_Audit_SOP_Review.xlsx
@@ -15,7 +15,7 @@
     <sheet name="DC" sheetId="5" state="visible" r:id="rId7"/>
     <sheet name="Dokumen" sheetId="6" state="visible" r:id="rId8"/>
     <sheet name="Pemetaan Medan-HO" sheetId="7" state="visible" r:id="rId9"/>
-    <sheet name="HO tanpa padanan Medan" sheetId="8" state="visible" r:id="rId10"/>
+    <sheet name="HO tidak ada di Medan" sheetId="8" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName function="false" hidden="false" localSheetId="4" name="_xlnm.Print_Titles" vbProcedure="false">DC!$1:$1</definedName>
@@ -23,7 +23,7 @@
     <definedName function="false" hidden="true" localSheetId="5" name="_xlnm._FilterDatabase" vbProcedure="false">Dokumen!$A$1:$I$134</definedName>
     <definedName function="false" hidden="false" localSheetId="1" name="_xlnm.Print_Titles" vbProcedure="false">Export!$1:$1</definedName>
     <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Export!$A$1:$P$63</definedName>
-    <definedName function="false" hidden="true" localSheetId="7" name="_xlnm._FilterDatabase" vbProcedure="false">'HO tanpa padanan Medan'!$A$1:$H$48</definedName>
+    <definedName function="false" hidden="true" localSheetId="7" name="_xlnm._FilterDatabase" vbProcedure="false">'HO tidak ada di Medan'!$A$1:$H$48</definedName>
     <definedName function="false" hidden="false" localSheetId="2" name="_xlnm.Print_Titles" vbProcedure="false">Import!$1:$1</definedName>
     <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">Import!$A$1:$P$73</definedName>
     <definedName function="false" hidden="true" localSheetId="6" name="_xlnm._FilterDatabase" vbProcedure="false">'Pemetaan Medan-HO'!$A$1:$N$171</definedName>
@@ -66,7 +66,7 @@
     <t xml:space="preserve">5. (TTD) berarti dokumen perlu tanda tangan. "(perkiraan)" berarti penempatan dokumen di tahap itu belum dipastikan.</t>
   </si>
   <si>
-    <t xml:space="preserve">6. Sheet "Pemetaan Medan-HO" memuat draf pemetaan 170 langkah SOP Medan ke SOP Utama HO, dan "HO tanpa padanan Medan" memuat langkah HO yang belum ada di SOP Medan. Isi kolom kuning untuk menyetujui atau mengubah padanan.</t>
+    <t xml:space="preserve">6. Sheet "Pemetaan Medan-HO" memuat draf pemetaan 170 langkah SOP Medan ke SOP Utama HO, dan "HO tidak ada di Medan" memuat langkah HO yang belum ada di SOP Medan. Isi kolom kuning untuk menyetujui atau mengubah pemetaan.</t>
   </si>
   <si>
     <t xml:space="preserve">7. Trucking Support langkah 1 sampai 8 (penarikan empty) asalnya Export 37 sampai 44. Langkah 9 sampai 22 (penarikan full container) belum diaudit dan masih draf dari Pendahuluan SOP.</t>
@@ -1764,16 +1764,16 @@
     <t xml:space="preserve">Langkah SOP Medan</t>
   </si>
   <si>
-    <t xml:space="preserve">Padanan di SOP HO</t>
+    <t xml:space="preserve">Sama dengan di SOP HO</t>
   </si>
   <si>
     <t xml:space="preserve">Langkah SOP HO</t>
   </si>
   <si>
-    <t xml:space="preserve">Relasi</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Keyakinan</t>
+    <t xml:space="preserve">Hubungan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kecocokan</t>
   </si>
   <si>
     <t xml:space="preserve">Catatan</t>
@@ -1782,7 +1782,7 @@
     <t xml:space="preserve">Setuju?</t>
   </si>
   <si>
-    <t xml:space="preserve">Padanan HO menurut reviewer</t>
+    <t xml:space="preserve">Langkah HO menurut reviewer</t>
   </si>
   <si>
     <t xml:space="preserve">MX1</t>
@@ -1797,7 +1797,7 @@
     <t xml:space="preserve">Export 3: Security registrasi, cek Surat Jalan, catat waktu tiba</t>
   </si>
   <si>
-    <t xml:space="preserve">sebagian</t>
+    <t xml:space="preserve">mirip</t>
   </si>
   <si>
     <t xml:space="preserve">sedang</t>
@@ -1824,10 +1824,10 @@
     <t xml:space="preserve">Export 2: Transporter registrasi kendaraan di Pos Security</t>
   </si>
   <si>
-    <t xml:space="preserve">setara</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Logbook Medan setara registrasi kendaraan di pos Security HO</t>
+    <t xml:space="preserve">sama</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Logbook Medan sama dengan registrasi kendaraan di pos Security HO</t>
   </si>
   <si>
     <t xml:space="preserve">Security arahkan supir lapor ke AO</t>
@@ -1896,10 +1896,10 @@
     <t xml:space="preserve">AO serahkan SJT; arahkan supir bayar uang bongkar ke Kasir</t>
   </si>
   <si>
-    <t xml:space="preserve">(tidak ada)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">hanya Medan</t>
+    <t xml:space="preserve">(tidak ada di HO)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hanya di Medan</t>
   </si>
   <si>
     <t xml:space="preserve">Uang bongkar dan Kasir tidak ada di SOP HO</t>
@@ -2103,7 +2103,7 @@
 Export 23: Admin serahkan copy CLP + Picking Report ke Picker</t>
   </si>
   <si>
-    <t xml:space="preserve">Stuffing list Medan setara CLP di HO</t>
+    <t xml:space="preserve">Stuffing list Medan sama dengan CLP di HO</t>
   </si>
   <si>
     <t xml:space="preserve">Checker/Operator</t>
@@ -2218,7 +2218,7 @@
     <t xml:space="preserve">Trucking 16: SPK ke vendor diterbitkan untuk penarikan ke CY UTPK/UTC</t>
   </si>
   <si>
-    <t xml:space="preserve">Pesan truck untuk full container ke pelabuhan setara SPK ke vendor</t>
+    <t xml:space="preserve">Pesan truck untuk full container ke pelabuhan sama dengan SPK ke vendor</t>
   </si>
   <si>
     <t xml:space="preserve">Operator RS/Supir</t>
@@ -2563,7 +2563,7 @@
     <t xml:space="preserve">Import 14: Trucking Support input gate in ke sistem; Security/Ops periksa kendaraan</t>
   </si>
   <si>
-    <t xml:space="preserve">Antar container ke CY MKT; HO langkah terdekat adalah input gate in</t>
+    <t xml:space="preserve">Antar container ke CY MKT; di HO langkah yang paling mirip adalah input gate in</t>
   </si>
   <si>
     <t xml:space="preserve">Supir/AO</t>
@@ -3034,7 +3034,7 @@
     <t xml:space="preserve">Export 10: Checker foto &amp; periksa segel dan nopol sebelum bongkar</t>
   </si>
   <si>
-    <t xml:space="preserve">Foto seal dan kondisi container; padanan terdekat ada di Export 10 (DC HO tidak punya)</t>
+    <t xml:space="preserve">Foto seal dan kondisi container; yang paling mirip ada di Export 10 (DC HO tidak punya)</t>
   </si>
   <si>
     <t xml:space="preserve">Checker periksa fisik, marking, jumlah vs PL; laporkan temuan</t>
@@ -19488,7 +19488,7 @@
       <c r="M126" s="17"/>
       <c r="N126" s="17"/>
     </row>
-    <row r="127" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="127" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A127" s="24" t="s">
         <v>27</v>
       </c>
@@ -20022,7 +20022,7 @@
       <c r="M141" s="17"/>
       <c r="N141" s="17"/>
     </row>
-    <row r="142" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="142" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A142" s="24" t="s">
         <v>27</v>
       </c>
@@ -20090,7 +20090,7 @@
       <c r="M143" s="17"/>
       <c r="N143" s="17"/>
     </row>
-    <row r="144" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="144" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A144" s="24" t="s">
         <v>27</v>
       </c>

</xml_diff>